<commit_message>
Feature stage (charges, groups, fragment orbitals), exclusions, atom-order and geometry checks in verify
</commit_message>
<xml_diff>
--- a/data/all_BE_values.xlsx
+++ b/data/all_BE_values.xlsx
@@ -716,11 +716,10 @@
         <v>-58.54199999989942</v>
       </c>
       <c r="C4" s="2">
-        <v>-49.415999999968335</v>
+        <v>-28.703</v>
       </c>
       <c r="D4" s="1">
-        <f>C4-B4</f>
-        <v>9.125999999931082</v>
+        <v>29.839</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
BE table: accept numbers stored as text and typographic minus; name bad cells; fix Q1_2 NH4
</commit_message>
<xml_diff>
--- a/data/all_BE_values.xlsx
+++ b/data/all_BE_values.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t>monomer</t>
   </si>
@@ -212,6 +212,9 @@
   </si>
   <si>
     <t>Q1_2</t>
+  </si>
+  <si>
+    <t>−28.413</t>
   </si>
   <si>
     <t>Q1_3</t>
@@ -1546,15 +1549,15 @@
       <c r="A63" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B63" s="1">
-        <v>-28.312999999150634</v>
+      <c r="B63" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B64" s="1">
         <v>-26.756000000052154</v>
@@ -1569,7 +1572,7 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B65" s="1"/>
       <c r="C65" s="1">
@@ -1579,7 +1582,7 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B66" s="1"/>
       <c r="C66" s="1">
@@ -1589,7 +1592,7 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B67" s="1">
         <v>-67.47999999951571</v>
@@ -1604,7 +1607,7 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B68" s="1">
         <v>-67.43799999915063</v>
@@ -1619,7 +1622,7 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B69" s="1">
         <v>-67.38499999977648</v>

</xml_diff>